<commit_message>
Step 6: Excel output
- app/render_excel.py fills templates/test_report.xlsx from a report: every
  cell exactly as the engine printed it, numbers stored as numbers with
  matching decimals, dates as dates shown dd-mm-yyyy, superscripts kept.
  One file per report or one combined workbook with a sheet per report.
- Signature placed after "Tested by :-".
- Template: "Tested by :-" moved to the right side, page centred on A4
  (sample margins were 0.59" left / 0" right), print area extended so the
  signature isn't cut off.
- tests/test_excel.py writes 33 real reports plus a combined workbook and
  checks every cell, layout, superscripts, page setup and signature.
</commit_message>
<xml_diff>
--- a/templates/test_report.xlsx
+++ b/templates/test_report.xlsx
@@ -9,7 +9,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Report" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'Test Report'!$A$1:$L$40</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'Test Report'!$A$1:$L$42</definedName>
   </definedNames>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
 </workbook>
@@ -8907,15 +8907,15 @@
       <c r="IV37" s="107" t="n"/>
     </row>
     <row r="39">
-      <c r="B39" s="111" t="inlineStr">
-        <is>
-          <t>Tested by :-</t>
-        </is>
-      </c>
+      <c r="B39" s="111" t="n"/>
       <c r="D39" s="111" t="n"/>
       <c r="E39" s="111" t="n"/>
       <c r="F39" s="111" t="n"/>
-      <c r="G39" s="111" t="n"/>
+      <c r="G39" s="111" t="inlineStr">
+        <is>
+          <t>Tested by :-</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="105">
@@ -9007,7 +9007,6 @@
     <mergeCell ref="J20:L20"/>
     <mergeCell ref="C26:C27"/>
     <mergeCell ref="G33:I33"/>
-    <mergeCell ref="B39:C39"/>
     <mergeCell ref="G15:L15"/>
     <mergeCell ref="J31:L31"/>
     <mergeCell ref="G35:I35"/>
@@ -9021,11 +9020,13 @@
     <mergeCell ref="D8:E8"/>
     <mergeCell ref="D19:F19"/>
     <mergeCell ref="A1:L1"/>
+    <mergeCell ref="G39:I39"/>
     <mergeCell ref="J18:K18"/>
     <mergeCell ref="C24:C25"/>
     <mergeCell ref="J17:K17"/>
   </mergeCells>
-  <pageMargins left="0.5905511811023623" right="0" top="0.2165354330708661" bottom="0" header="0.2362204724409449" footer="0.3149606299212598"/>
+  <printOptions horizontalCentered="1"/>
+  <pageMargins left="0.4" right="0.4" top="0.2165354330708661" bottom="0" header="0.2362204724409449" footer="0.3149606299212598"/>
   <pageSetup orientation="portrait" paperSize="9" fitToHeight="1" fitToWidth="1" verticalDpi="200"/>
 </worksheet>
 </file>
</xml_diff>